<commit_message>
Enhance login and results page functionality; add new inspection scripts for Amazon product interactions
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -28,6 +28,7 @@
     <sheet name="sheet516" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="sheet517" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="sheet518" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="sheet519" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -845,6 +846,27 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: Add Allure report files for test results and metrics
- Created JSON files for individual test cases and timeline data.
- Added InfluxDB and Prometheus export files for launch metrics.
- Implemented HTML mail template for report summary.
- Generated history and trend JSON files for test results.
- Established widgets for displaying various statistics in the Allure report.
- Included summary JSON for overall test run statistics.
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -29,6 +29,7 @@
     <sheet name="sheet517" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="sheet518" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="sheet519" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="sheet520" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -867,6 +868,27 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
chore: Update sample credentials file for testing
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -30,6 +30,7 @@
     <sheet name="sheet518" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="sheet519" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="sheet520" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="sheet521" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -889,6 +890,27 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: Enhance test steps with detailed Allure reporting and improve CI workflow
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -31,6 +31,10 @@
     <sheet name="sheet519" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="sheet520" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="sheet521" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="sheet522" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="sheet523" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="sheet524" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="sheet525" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -911,6 +915,90 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: Update browser launch configuration to headless mode and add new Amazon test script for product search and cart count verification
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -35,6 +35,7 @@
     <sheet name="sheet523" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="sheet524" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="sheet525" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="sheet526" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1073,6 +1074,27 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add new test cases for data handling and login functionality
- Created JSON reports for the following test cases:
  - test_positiveLogin for successful login scenario
  - test_json_1 for JSON data handling
  - test_cli_env for command line environment testing
  - test_csv for CSV data handling
  - test_sum for summation functionality with parameters
</commit_message>
<xml_diff>
--- a/testData/sample_creds.xlsx
+++ b/testData/sample_creds.xlsx
@@ -36,6 +36,7 @@
     <sheet name="sheet524" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="sheet525" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="sheet526" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="sheet527" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1095,6 +1096,27 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>